<commit_message>
Enhance logging configuration and messages for improved clarity; update chunk size in CSV reader for better performance
</commit_message>
<xml_diff>
--- a/outputs/anomaly_reports.xlsx
+++ b/outputs/anomaly_reports.xlsx
@@ -12,6 +12,7 @@
     <sheet name="By_Sector" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="By_Group" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="By_Sector_&amp;_Group" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Missing_Data_Analysis" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -572,31 +573,31 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2014</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Chemical industry</t>
+          <t>Production and processing of metals</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Sandoz GmbH</t>
+          <t>voestalpine Stahl GmbH</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Hydrochlorofluorocarbons (HCFCs)</t>
+          <t>Carbon dioxide (CO2)</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>10</v>
+        <v>8500000000</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -607,37 +608,37 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>2.397895272798371</v>
+        <v>22.86333200056033</v>
       </c>
       <c r="K2" t="n">
         <v>19.08593942191924</v>
       </c>
       <c r="L2" t="n">
-        <v>-16.68804414912086</v>
+        <v>3.777392578641095</v>
       </c>
       <c r="M2" t="n">
-        <v>12.19095120020471</v>
+        <v>8.677774453654962</v>
       </c>
       <c r="N2" t="n">
-        <v>-9.793055927406341</v>
+        <v>14.18555754690537</v>
       </c>
       <c r="O2" t="n">
-        <v>12.83601552677931</v>
+        <v>21.81518913779929</v>
       </c>
       <c r="P2" t="n">
-        <v>-10.43812025398094</v>
+        <v>1.048142862761036</v>
       </c>
       <c r="Q2" t="n">
-        <v>341</v>
+        <v>291000000</v>
       </c>
       <c r="R2" t="n">
-        <v>-97.0674486803519</v>
+        <v>2820.962199312715</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
       </c>
       <c r="T2" t="n">
-        <v>-0.1290983602935629</v>
+        <v>-0.1904606211191381</v>
       </c>
     </row>
     <row r="3">
@@ -648,7 +649,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2007</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -672,7 +673,7 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>8730000000</v>
+        <v>9340000000</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -683,37 +684,37 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>22.89003120691247</v>
+        <v>22.95757208929423</v>
       </c>
       <c r="K3" t="n">
         <v>19.08593942191924</v>
       </c>
       <c r="L3" t="n">
-        <v>3.804091784993233</v>
+        <v>3.871632667374993</v>
       </c>
       <c r="M3" t="n">
         <v>8.677774453654962</v>
       </c>
       <c r="N3" t="n">
-        <v>14.21225675325751</v>
+        <v>14.27979763563927</v>
       </c>
       <c r="O3" t="n">
         <v>21.81518913779929</v>
       </c>
       <c r="P3" t="n">
-        <v>1.074842069113174</v>
+        <v>1.142382951494934</v>
       </c>
       <c r="Q3" t="n">
-        <v>329000000</v>
+        <v>318000000</v>
       </c>
       <c r="R3" t="n">
-        <v>2553.495440729484</v>
+        <v>2837.106918238994</v>
       </c>
       <c r="S3" t="n">
         <v>1</v>
       </c>
       <c r="T3" t="n">
-        <v>-0.1104180954378707</v>
+        <v>-0.1899441665546868</v>
       </c>
     </row>
     <row r="4">
@@ -724,7 +725,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2012</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -748,7 +749,7 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>8810000000</v>
+        <v>8440000000</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -759,37 +760,37 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>22.89915327700801</v>
+        <v>22.85624814567276</v>
       </c>
       <c r="K4" t="n">
         <v>19.08593942191924</v>
       </c>
       <c r="L4" t="n">
-        <v>3.813213855088772</v>
+        <v>3.770308723753526</v>
       </c>
       <c r="M4" t="n">
         <v>8.677774453654962</v>
       </c>
       <c r="N4" t="n">
-        <v>14.22137882335305</v>
+        <v>14.1784736920178</v>
       </c>
       <c r="O4" t="n">
         <v>21.81518913779929</v>
       </c>
       <c r="P4" t="n">
-        <v>1.083964139208714</v>
+        <v>1.041059007873468</v>
       </c>
       <c r="Q4" t="n">
-        <v>330000000</v>
+        <v>303000000</v>
       </c>
       <c r="R4" t="n">
-        <v>2569.69696969697</v>
+        <v>2685.478547854786</v>
       </c>
       <c r="S4" t="n">
         <v>1</v>
       </c>
       <c r="T4" t="n">
-        <v>-0.1104180954378707</v>
+        <v>-0.1894280612981443</v>
       </c>
     </row>
     <row r="5">
@@ -800,7 +801,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2009</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -824,7 +825,7 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>6880000000</v>
+        <v>8560000000</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -835,37 +836,37 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>22.65188448903701</v>
+        <v>22.87036602721689</v>
       </c>
       <c r="K5" t="n">
         <v>19.08593942191924</v>
       </c>
       <c r="L5" t="n">
-        <v>3.565945067117777</v>
+        <v>3.78442660529765</v>
       </c>
       <c r="M5" t="n">
         <v>8.677774453654962</v>
       </c>
       <c r="N5" t="n">
-        <v>13.97411003538205</v>
+        <v>14.19259157356192</v>
       </c>
       <c r="O5" t="n">
         <v>21.81518913779929</v>
       </c>
       <c r="P5" t="n">
-        <v>0.8366953512377187</v>
+        <v>1.055176889417591</v>
       </c>
       <c r="Q5" t="n">
-        <v>259000000</v>
+        <v>311000000</v>
       </c>
       <c r="R5" t="n">
-        <v>2556.370656370656</v>
+        <v>2652.411575562701</v>
       </c>
       <c r="S5" t="n">
         <v>1</v>
       </c>
       <c r="T5" t="n">
-        <v>-0.1077034019325231</v>
+        <v>-0.1894280612981443</v>
       </c>
     </row>
     <row r="6">
@@ -876,7 +877,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2013</t>
+          <t>2018</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -900,7 +901,7 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>8600000000</v>
+        <v>7750000000</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -911,37 +912,37 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>22.87502804032215</v>
+        <v>22.7709586804407</v>
       </c>
       <c r="K6" t="n">
         <v>19.08593942191924</v>
       </c>
       <c r="L6" t="n">
-        <v>3.789088618402918</v>
+        <v>3.685019258521464</v>
       </c>
       <c r="M6" t="n">
         <v>8.677774453654962</v>
       </c>
       <c r="N6" t="n">
-        <v>14.19725358666719</v>
+        <v>14.09318422678574</v>
       </c>
       <c r="O6" t="n">
         <v>21.81518913779929</v>
       </c>
       <c r="P6" t="n">
-        <v>1.059838902522859</v>
+        <v>0.9557695426414057</v>
       </c>
       <c r="Q6" t="n">
-        <v>371000000</v>
+        <v>274000000</v>
       </c>
       <c r="R6" t="n">
-        <v>2218.059299191375</v>
+        <v>2728.467153284671</v>
       </c>
       <c r="S6" t="n">
         <v>1</v>
       </c>
       <c r="T6" t="n">
-        <v>-0.1066580129545179</v>
+        <v>-0.1863387520057622</v>
       </c>
     </row>
     <row r="7">
@@ -952,7 +953,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2014</t>
+          <t>2007</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -976,7 +977,7 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>8660000000</v>
+        <v>8730000000</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -987,37 +988,37 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>22.88198055963623</v>
+        <v>22.89003120691247</v>
       </c>
       <c r="K7" t="n">
         <v>19.08593942191924</v>
       </c>
       <c r="L7" t="n">
-        <v>3.796041137716994</v>
+        <v>3.804091784993233</v>
       </c>
       <c r="M7" t="n">
         <v>8.677774453654962</v>
       </c>
       <c r="N7" t="n">
-        <v>14.20420610598127</v>
+        <v>14.21225675325751</v>
       </c>
       <c r="O7" t="n">
         <v>21.81518913779929</v>
       </c>
       <c r="P7" t="n">
-        <v>1.066791421836935</v>
+        <v>1.074842069113174</v>
       </c>
       <c r="Q7" t="n">
-        <v>370000000</v>
+        <v>329000000</v>
       </c>
       <c r="R7" t="n">
-        <v>2240.540540540541</v>
+        <v>2553.495440729484</v>
       </c>
       <c r="S7" t="n">
         <v>1</v>
       </c>
       <c r="T7" t="n">
-        <v>-0.1066580129545179</v>
+        <v>-0.1853117660132111</v>
       </c>
     </row>
     <row r="8">
@@ -1028,7 +1029,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1052,7 +1053,7 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>9340000000</v>
+        <v>8810000000</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -1063,37 +1064,37 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>22.95757208929423</v>
+        <v>22.89915327700801</v>
       </c>
       <c r="K8" t="n">
         <v>19.08593942191924</v>
       </c>
       <c r="L8" t="n">
-        <v>3.871632667374993</v>
+        <v>3.813213855088772</v>
       </c>
       <c r="M8" t="n">
         <v>8.677774453654962</v>
       </c>
       <c r="N8" t="n">
-        <v>14.27979763563927</v>
+        <v>14.22137882335305</v>
       </c>
       <c r="O8" t="n">
         <v>21.81518913779929</v>
       </c>
       <c r="P8" t="n">
-        <v>1.142382951494934</v>
+        <v>1.083964139208714</v>
       </c>
       <c r="Q8" t="n">
-        <v>318000000</v>
+        <v>330000000</v>
       </c>
       <c r="R8" t="n">
-        <v>2837.106918238994</v>
+        <v>2569.69696969697</v>
       </c>
       <c r="S8" t="n">
         <v>1</v>
       </c>
       <c r="T8" t="n">
-        <v>-0.1062150411920125</v>
+        <v>-0.1853117660132111</v>
       </c>
     </row>
     <row r="9">
@@ -1104,7 +1105,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2015</t>
+          <t>2011</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1128,7 +1129,7 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>8640000000</v>
+        <v>8470000000</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -1139,37 +1140,37 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>22.87966841987812</v>
+        <v>22.85979634572844</v>
       </c>
       <c r="K9" t="n">
         <v>19.08593942191924</v>
       </c>
       <c r="L9" t="n">
-        <v>3.79372899795888</v>
+        <v>3.773856923809202</v>
       </c>
       <c r="M9" t="n">
         <v>8.677774453654962</v>
       </c>
       <c r="N9" t="n">
-        <v>14.20189396622315</v>
+        <v>14.18202189207348</v>
       </c>
       <c r="O9" t="n">
         <v>21.81518913779929</v>
       </c>
       <c r="P9" t="n">
-        <v>1.064479282078821</v>
+        <v>1.044607207929143</v>
       </c>
       <c r="Q9" t="n">
-        <v>366000000</v>
+        <v>340000000</v>
       </c>
       <c r="R9" t="n">
-        <v>2260.655737704918</v>
+        <v>2391.176470588235</v>
       </c>
       <c r="S9" t="n">
         <v>1</v>
       </c>
       <c r="T9" t="n">
-        <v>-0.1062073415499674</v>
+        <v>-0.1827503727036507</v>
       </c>
     </row>
     <row r="10">
@@ -1180,31 +1181,31 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2010</t>
+          <t>2009</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Chemical industry</t>
+          <t>Production and processing of metals</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Patheon Austria GmbH &amp; Co KG</t>
+          <t>voestalpine Stahl GmbH</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Hydrochlorofluorocarbons (HCFCs)</t>
+          <t>Carbon dioxide (CO2)</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>36</v>
+        <v>6880000000</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -1215,37 +1216,37 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>3.610917912644224</v>
+        <v>22.65188448903701</v>
       </c>
       <c r="K10" t="n">
         <v>19.08593942191924</v>
       </c>
       <c r="L10" t="n">
-        <v>-15.47502150927501</v>
+        <v>3.565945067117777</v>
       </c>
       <c r="M10" t="n">
-        <v>12.19095120020471</v>
+        <v>8.677774453654962</v>
       </c>
       <c r="N10" t="n">
-        <v>-8.580033287560488</v>
+        <v>13.97411003538205</v>
       </c>
       <c r="O10" t="n">
-        <v>12.83601552677931</v>
+        <v>21.81518913779929</v>
       </c>
       <c r="P10" t="n">
-        <v>-9.225097614135088</v>
+        <v>0.8366953512377187</v>
       </c>
       <c r="Q10" t="n">
-        <v>600</v>
+        <v>259000000</v>
       </c>
       <c r="R10" t="n">
-        <v>-94</v>
+        <v>2556.370656370656</v>
       </c>
       <c r="S10" t="n">
         <v>1</v>
       </c>
       <c r="T10" t="n">
-        <v>-0.1059802598225257</v>
+        <v>-0.1827382704483099</v>
       </c>
     </row>
     <row r="11">
@@ -1256,7 +1257,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2011</t>
+          <t>2015</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1280,7 +1281,7 @@
         </is>
       </c>
       <c r="G11" t="n">
-        <v>8470000000</v>
+        <v>8640000000</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -1291,37 +1292,37 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>22.85979634572844</v>
+        <v>22.87966841987812</v>
       </c>
       <c r="K11" t="n">
         <v>19.08593942191924</v>
       </c>
       <c r="L11" t="n">
-        <v>3.773856923809202</v>
+        <v>3.79372899795888</v>
       </c>
       <c r="M11" t="n">
         <v>8.677774453654962</v>
       </c>
       <c r="N11" t="n">
-        <v>14.18202189207348</v>
+        <v>14.20189396622315</v>
       </c>
       <c r="O11" t="n">
         <v>21.81518913779929</v>
       </c>
       <c r="P11" t="n">
-        <v>1.044607207929143</v>
+        <v>1.064479282078821</v>
       </c>
       <c r="Q11" t="n">
-        <v>340000000</v>
+        <v>366000000</v>
       </c>
       <c r="R11" t="n">
-        <v>2391.176470588235</v>
+        <v>2260.655737704918</v>
       </c>
       <c r="S11" t="n">
         <v>1</v>
       </c>
       <c r="T11" t="n">
-        <v>-0.1058890627014608</v>
+        <v>-0.179688116658861</v>
       </c>
     </row>
     <row r="12">
@@ -1397,7 +1398,7 @@
         <v>1</v>
       </c>
       <c r="T12" t="n">
-        <v>-0.1057569749603933</v>
+        <v>-0.179178948158403</v>
       </c>
     </row>
     <row r="13">
@@ -1408,7 +1409,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2012</t>
+          <t>2013</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1432,7 +1433,7 @@
         </is>
       </c>
       <c r="G13" t="n">
-        <v>8440000000</v>
+        <v>8600000000</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -1443,37 +1444,37 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>22.85624814567276</v>
+        <v>22.87502804032215</v>
       </c>
       <c r="K13" t="n">
         <v>19.08593942191924</v>
       </c>
       <c r="L13" t="n">
-        <v>3.770308723753526</v>
+        <v>3.789088618402918</v>
       </c>
       <c r="M13" t="n">
         <v>8.677774453654962</v>
       </c>
       <c r="N13" t="n">
-        <v>14.1784736920178</v>
+        <v>14.19725358666719</v>
       </c>
       <c r="O13" t="n">
         <v>21.81518913779929</v>
       </c>
       <c r="P13" t="n">
-        <v>1.041059007873468</v>
+        <v>1.059838902522859</v>
       </c>
       <c r="Q13" t="n">
-        <v>303000000</v>
+        <v>371000000</v>
       </c>
       <c r="R13" t="n">
-        <v>2685.478547854786</v>
+        <v>2218.059299191375</v>
       </c>
       <c r="S13" t="n">
         <v>1</v>
       </c>
       <c r="T13" t="n">
-        <v>-0.1054617496974416</v>
+        <v>-0.17867012403787</v>
       </c>
     </row>
     <row r="14">
@@ -1484,7 +1485,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2014</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1508,7 +1509,7 @@
         </is>
       </c>
       <c r="G14" t="n">
-        <v>8500000000</v>
+        <v>8660000000</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -1519,37 +1520,37 @@
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>22.86333200056033</v>
+        <v>22.88198055963623</v>
       </c>
       <c r="K14" t="n">
         <v>19.08593942191924</v>
       </c>
       <c r="L14" t="n">
-        <v>3.777392578641095</v>
+        <v>3.796041137716994</v>
       </c>
       <c r="M14" t="n">
         <v>8.677774453654962</v>
       </c>
       <c r="N14" t="n">
-        <v>14.18555754690537</v>
+        <v>14.20420610598127</v>
       </c>
       <c r="O14" t="n">
         <v>21.81518913779929</v>
       </c>
       <c r="P14" t="n">
-        <v>1.048142862761036</v>
+        <v>1.066791421836935</v>
       </c>
       <c r="Q14" t="n">
-        <v>291000000</v>
+        <v>370000000</v>
       </c>
       <c r="R14" t="n">
-        <v>2820.962199312715</v>
+        <v>2240.540540540541</v>
       </c>
       <c r="S14" t="n">
         <v>1</v>
       </c>
       <c r="T14" t="n">
-        <v>-0.1054617496974416</v>
+        <v>-0.17867012403787</v>
       </c>
     </row>
     <row r="15">
@@ -1560,31 +1561,31 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2014</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Production and processing of metals</t>
+          <t>Chemical industry</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>voestalpine Stahl GmbH</t>
+          <t>Sandoz GmbH</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Carbon dioxide (CO2)</t>
+          <t>Hydrochlorofluorocarbons (HCFCs)</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>8560000000</v>
+        <v>623</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -1595,37 +1596,37 @@
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>22.87036602721689</v>
+        <v>6.436150368369428</v>
       </c>
       <c r="K15" t="n">
         <v>19.08593942191924</v>
       </c>
       <c r="L15" t="n">
-        <v>3.78442660529765</v>
+        <v>-12.64978905354981</v>
       </c>
       <c r="M15" t="n">
-        <v>8.677774453654962</v>
+        <v>12.19095120020471</v>
       </c>
       <c r="N15" t="n">
-        <v>14.19259157356192</v>
+        <v>-5.754800831835284</v>
       </c>
       <c r="O15" t="n">
-        <v>21.81518913779929</v>
+        <v>12.83601552677931</v>
       </c>
       <c r="P15" t="n">
-        <v>1.055176889417591</v>
+        <v>-6.399865158409884</v>
       </c>
       <c r="Q15" t="n">
-        <v>311000000</v>
+        <v>10</v>
       </c>
       <c r="R15" t="n">
-        <v>2652.411575562701</v>
+        <v>6130</v>
       </c>
       <c r="S15" t="n">
         <v>1</v>
       </c>
       <c r="T15" t="n">
-        <v>-0.1050118873944956</v>
+        <v>-0.1624277032504617</v>
       </c>
     </row>
     <row r="16">
@@ -1636,31 +1637,31 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2014</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Production and processing of metals</t>
+          <t>Chemical industry</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>voestalpine Stahl GmbH</t>
+          <t>Sandoz GmbH</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Carbon dioxide (CO2)</t>
+          <t>Hydrochlorofluorocarbons (HCFCs)</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>7750000000</v>
+        <v>10</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -1671,37 +1672,37 @@
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>22.7709586804407</v>
+        <v>2.397895272798371</v>
       </c>
       <c r="K16" t="n">
         <v>19.08593942191924</v>
       </c>
       <c r="L16" t="n">
-        <v>3.685019258521464</v>
+        <v>-16.68804414912086</v>
       </c>
       <c r="M16" t="n">
-        <v>8.677774453654962</v>
+        <v>12.19095120020471</v>
       </c>
       <c r="N16" t="n">
-        <v>14.09318422678574</v>
+        <v>-9.793055927406341</v>
       </c>
       <c r="O16" t="n">
-        <v>21.81518913779929</v>
+        <v>12.83601552677931</v>
       </c>
       <c r="P16" t="n">
-        <v>0.9557695426414057</v>
+        <v>-10.43812025398094</v>
       </c>
       <c r="Q16" t="n">
-        <v>274000000</v>
+        <v>341</v>
       </c>
       <c r="R16" t="n">
-        <v>2728.467153284671</v>
+        <v>-97.0674486803519</v>
       </c>
       <c r="S16" t="n">
         <v>1</v>
       </c>
       <c r="T16" t="n">
-        <v>-0.1045623293592841</v>
+        <v>-0.1294002393881796</v>
       </c>
     </row>
     <row r="17">
@@ -1712,72 +1713,72 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2010</t>
+          <t>2018</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Energy sector</t>
+          <t>Mineral industry</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>OMV Downstream GmbH</t>
+          <t>Leube Zement GmbH</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Hydrochlorofluorocarbons (HCFCs)</t>
+          <t>Naphthalene</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>147</v>
+        <v>1140</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Regulated Climate/Ozone Risk - Global Environmental Impact</t>
+          <t>High Risk - Persistent Toxins, Carcinogens &amp; Long-Term Illness</t>
         </is>
       </c>
       <c r="I17" t="b">
         <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>4.997212273764115</v>
+        <v>7.039660349862076</v>
       </c>
       <c r="K17" t="n">
-        <v>19.08593942191924</v>
+        <v>4.923617305492665</v>
       </c>
       <c r="L17" t="n">
-        <v>-14.08872714815512</v>
+        <v>2.116043044369411</v>
       </c>
       <c r="M17" t="n">
-        <v>13.27250775700296</v>
+        <v>12.68230993011178</v>
       </c>
       <c r="N17" t="n">
-        <v>-8.275295483238848</v>
+        <v>-5.642649580249709</v>
       </c>
       <c r="O17" t="n">
-        <v>18.95130900089689</v>
+        <v>4.870484311519177</v>
       </c>
       <c r="P17" t="n">
-        <v>-13.95409672713277</v>
+        <v>2.169176038342899</v>
       </c>
       <c r="Q17" t="n">
-        <v>345</v>
+        <v>101</v>
       </c>
       <c r="R17" t="n">
-        <v>-57.39130434782609</v>
+        <v>1028.712871287129</v>
       </c>
       <c r="S17" t="n">
         <v>1</v>
       </c>
       <c r="T17" t="n">
-        <v>-0.1023007468251805</v>
+        <v>-0.1024886395961313</v>
       </c>
     </row>
     <row r="18">
@@ -1788,7 +1789,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2013</t>
+          <t>2010</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1812,7 +1813,7 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -1823,37 +1824,37 @@
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>3.258096538021482</v>
+        <v>3.610917912644224</v>
       </c>
       <c r="K18" t="n">
         <v>19.08593942191924</v>
       </c>
       <c r="L18" t="n">
-        <v>-15.82784288389775</v>
+        <v>-15.47502150927501</v>
       </c>
       <c r="M18" t="n">
         <v>12.19095120020471</v>
       </c>
       <c r="N18" t="n">
-        <v>-8.93285466218323</v>
+        <v>-8.580033287560488</v>
       </c>
       <c r="O18" t="n">
         <v>12.83601552677931</v>
       </c>
       <c r="P18" t="n">
-        <v>-9.57791898875783</v>
+        <v>-9.225097614135088</v>
       </c>
       <c r="Q18" t="n">
-        <v>41</v>
+        <v>600</v>
       </c>
       <c r="R18" t="n">
-        <v>-39.02439024390244</v>
+        <v>-94</v>
       </c>
       <c r="S18" t="n">
         <v>1</v>
       </c>
       <c r="T18" t="n">
-        <v>-0.0983893057312113</v>
+        <v>-0.1021735843681947</v>
       </c>
     </row>
     <row r="19">
@@ -1864,22 +1865,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2012</t>
+          <t>2010</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Chemical industry</t>
+          <t>Energy sector</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Patheon Austria GmbH &amp; Co KG</t>
+          <t>OMV Downstream GmbH</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1888,7 +1889,7 @@
         </is>
       </c>
       <c r="G19" t="n">
-        <v>41</v>
+        <v>147</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -1899,37 +1900,37 @@
         <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>3.737669618283368</v>
+        <v>4.997212273764115</v>
       </c>
       <c r="K19" t="n">
         <v>19.08593942191924</v>
       </c>
       <c r="L19" t="n">
-        <v>-15.34826980363587</v>
+        <v>-14.08872714815512</v>
       </c>
       <c r="M19" t="n">
-        <v>12.19095120020471</v>
+        <v>13.27250775700296</v>
       </c>
       <c r="N19" t="n">
-        <v>-8.453281581921344</v>
+        <v>-8.275295483238848</v>
       </c>
       <c r="O19" t="n">
-        <v>12.83601552677931</v>
+        <v>18.95130900089689</v>
       </c>
       <c r="P19" t="n">
-        <v>-9.098345908495943</v>
+        <v>-13.95409672713277</v>
       </c>
       <c r="Q19" t="n">
-        <v>36</v>
+        <v>345</v>
       </c>
       <c r="R19" t="n">
-        <v>13.88888888888889</v>
+        <v>-57.39130434782609</v>
       </c>
       <c r="S19" t="n">
         <v>1</v>
       </c>
       <c r="T19" t="n">
-        <v>-0.09091901784504897</v>
+        <v>-0.09401107019937116</v>
       </c>
     </row>
     <row r="20">
@@ -1940,31 +1941,31 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2010</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Chemical industry</t>
+          <t>Energy sector</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Sandoz GmbH</t>
+          <t>WIEN ENERGIE GmbH</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Hydro-fluorocarbons (HFCS)</t>
+          <t>Carbon dioxide (CO2)</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>104</v>
+        <v>1960000000</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -1975,37 +1976,37 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>4.653960350157523</v>
+        <v>21.39621031069904</v>
       </c>
       <c r="K20" t="n">
         <v>19.08593942191924</v>
       </c>
       <c r="L20" t="n">
-        <v>-14.43197907176171</v>
+        <v>2.310270888779804</v>
       </c>
       <c r="M20" t="n">
-        <v>12.19095120020471</v>
+        <v>13.27250775700296</v>
       </c>
       <c r="N20" t="n">
-        <v>-7.536990850047188</v>
+        <v>8.123702553696077</v>
       </c>
       <c r="O20" t="n">
-        <v>12.83601552677931</v>
+        <v>18.95130900089689</v>
       </c>
       <c r="P20" t="n">
-        <v>-8.182055176621787</v>
+        <v>2.444901309802152</v>
       </c>
       <c r="Q20" t="n">
-        <v>232</v>
+        <v>192000000</v>
       </c>
       <c r="R20" t="n">
-        <v>-55.17241379310344</v>
+        <v>920.8333333333334</v>
       </c>
       <c r="S20" t="n">
         <v>1</v>
       </c>
       <c r="T20" t="n">
-        <v>-0.08794063032443478</v>
+        <v>-0.08997761986909603</v>
       </c>
     </row>
     <row r="21">
@@ -2016,72 +2017,72 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2013</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Production and processing of metals</t>
+          <t>Chemical industry</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>voestalpine Stahl GmbH</t>
+          <t>Patheon Austria GmbH &amp; Co KG</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>PCDD + PCDF (dioxins + furans) (as Teq)</t>
+          <t>Hydrochlorofluorocarbons (HCFCs)</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>0.000199</v>
+        <v>25</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Critical Risk - Immediate Toxicity &amp; Severe Health Damage</t>
+          <t>Regulated Climate/Ozone Risk - Global Environmental Impact</t>
         </is>
       </c>
       <c r="I21" t="b">
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>0.0001989802021264743</v>
+        <v>3.258096538021482</v>
       </c>
       <c r="K21" t="n">
-        <v>3.796006532848082</v>
+        <v>19.08593942191924</v>
       </c>
       <c r="L21" t="n">
-        <v>-3.795807552645956</v>
+        <v>-15.82784288389775</v>
       </c>
       <c r="M21" t="n">
-        <v>8.677774453654962</v>
+        <v>12.19095120020471</v>
       </c>
       <c r="N21" t="n">
-        <v>-8.677575473452835</v>
+        <v>-8.93285466218323</v>
       </c>
       <c r="O21" t="n">
-        <v>5.398162701517752</v>
+        <v>12.83601552677931</v>
       </c>
       <c r="P21" t="n">
-        <v>-5.397963721315626</v>
+        <v>-9.57791898875783</v>
       </c>
       <c r="Q21" t="n">
-        <v>0.00104</v>
+        <v>41</v>
       </c>
       <c r="R21" t="n">
-        <v>-80.86538461538461</v>
+        <v>-39.02439024390244</v>
       </c>
       <c r="S21" t="n">
         <v>1</v>
       </c>
       <c r="T21" t="n">
-        <v>-0.08687859370045625</v>
+        <v>-0.08864713343244413</v>
       </c>
     </row>
   </sheetData>
@@ -2117,7 +2118,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3">
@@ -2127,7 +2128,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4">
@@ -2137,7 +2138,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5">
@@ -2147,13 +2148,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Other activities</t>
+          <t>Waste and wastewater management</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -2163,11 +2164,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Waste and wastewater management</t>
+          <t>Other activities</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2203,7 +2204,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>101</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3">
@@ -2213,7 +2214,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4">
@@ -2223,7 +2224,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5">
@@ -2279,7 +2280,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3">
@@ -2309,7 +2310,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5">
@@ -2324,7 +2325,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6">
@@ -2345,27 +2346,27 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Mineral industry</t>
+          <t>Waste and wastewater management</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Critical Risk - Immediate Toxicity &amp; Severe Health Damage</t>
+          <t>Regulated Climate/Ozone Risk - Global Environmental Impact</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Other activities</t>
+          <t>Mineral industry</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Regulated Climate/Ozone Risk - Global Environmental Impact</t>
+          <t>Critical Risk - Immediate Toxicity &amp; Severe Health Damage</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -2375,12 +2376,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Waste and wastewater management</t>
+          <t>Mineral industry</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Regulated Climate/Ozone Risk - Global Environmental Impact</t>
+          <t>Moderate Risk - Air Pollution, Corrosives &amp; Community Exposure</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -2390,7 +2391,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Chemical industry</t>
+          <t>Energy sector</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2405,12 +2406,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Mineral industry</t>
+          <t>Other activities</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Moderate Risk - Air Pollution, Corrosives &amp; Community Exposure</t>
+          <t>Regulated Climate/Ozone Risk - Global Environmental Impact</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -2430,6 +2431,240 @@
       </c>
       <c r="C12" t="n">
         <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>missing_values</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>missing_percent</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>confidentialityReason</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>372128</v>
+      </c>
+      <c r="C2" t="n">
+        <v>99.97904386280716</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>addressConfidentialityReason</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>371400</v>
+      </c>
+      <c r="C3" t="n">
+        <v>99.78345324900727</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>EPRTR_SectorCode</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>4985</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1.339312101363223</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>EPRTR_SectorName</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4985</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1.339312101363223</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>EPRTRAnnexIMainActivity</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>4985</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1.339312101363223</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Latitude</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>806</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.2165467509927298</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Longitude</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>806</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.2165467509927298</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>city</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>133</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.03573290059805592</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Releases</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>78</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.02095613719284482</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>facilityName</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.0002686684255492926</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>countryName</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>reportingYear</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>FacilityInspireId</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>PublicationDate</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Pollutant</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>TargetRelease</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactor model training process to include train-test split; update anomaly prediction logic and score assignment
</commit_message>
<xml_diff>
--- a/outputs/anomaly_reports.xlsx
+++ b/outputs/anomaly_reports.xlsx
@@ -595,7 +595,7 @@
         <v>1</v>
       </c>
       <c r="T2" t="n">
-        <v>-0.1904606211191381</v>
+        <v>-0.1689634045385567</v>
       </c>
     </row>
     <row r="3">
@@ -606,7 +606,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2012</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -630,7 +630,7 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>9340000000</v>
+        <v>8440000000</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -641,37 +641,37 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>22.95757208929423</v>
+        <v>22.85624814567276</v>
       </c>
       <c r="K3" t="n">
         <v>19.08593942191924</v>
       </c>
       <c r="L3" t="n">
-        <v>3.871632667374993</v>
+        <v>3.770308723753526</v>
       </c>
       <c r="M3" t="n">
         <v>8.677774453654962</v>
       </c>
       <c r="N3" t="n">
-        <v>14.27979763563927</v>
+        <v>14.1784736920178</v>
       </c>
       <c r="O3" t="n">
         <v>21.81518913779929</v>
       </c>
       <c r="P3" t="n">
-        <v>1.142382951494934</v>
+        <v>1.041059007873468</v>
       </c>
       <c r="Q3" t="n">
-        <v>318000000</v>
+        <v>303000000</v>
       </c>
       <c r="R3" t="n">
-        <v>2837.106918238994</v>
+        <v>2685.478547854786</v>
       </c>
       <c r="S3" t="n">
         <v>1</v>
       </c>
       <c r="T3" t="n">
-        <v>-0.1899441665546868</v>
+        <v>-0.1689634045385567</v>
       </c>
     </row>
     <row r="4">
@@ -682,7 +682,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2012</t>
+          <t>2016</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>8440000000</v>
+        <v>8600000000</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -717,37 +717,37 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>22.85624814567276</v>
+        <v>22.87502804032215</v>
       </c>
       <c r="K4" t="n">
         <v>19.08593942191924</v>
       </c>
       <c r="L4" t="n">
-        <v>3.770308723753526</v>
+        <v>3.789088618402918</v>
       </c>
       <c r="M4" t="n">
         <v>8.677774453654962</v>
       </c>
       <c r="N4" t="n">
-        <v>14.1784736920178</v>
+        <v>14.19725358666719</v>
       </c>
       <c r="O4" t="n">
         <v>21.81518913779929</v>
       </c>
       <c r="P4" t="n">
-        <v>1.041059007873468</v>
+        <v>1.059838902522859</v>
       </c>
       <c r="Q4" t="n">
-        <v>303000000</v>
+        <v>362000000</v>
       </c>
       <c r="R4" t="n">
-        <v>2685.478547854786</v>
+        <v>2275.690607734807</v>
       </c>
       <c r="S4" t="n">
         <v>1</v>
       </c>
       <c r="T4" t="n">
-        <v>-0.1894280612981443</v>
+        <v>-0.1669568187097168</v>
       </c>
     </row>
     <row r="5">
@@ -758,7 +758,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2011</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -782,7 +782,7 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>8560000000</v>
+        <v>8470000000</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -793,37 +793,37 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>22.87036602721689</v>
+        <v>22.85979634572844</v>
       </c>
       <c r="K5" t="n">
         <v>19.08593942191924</v>
       </c>
       <c r="L5" t="n">
-        <v>3.78442660529765</v>
+        <v>3.773856923809202</v>
       </c>
       <c r="M5" t="n">
         <v>8.677774453654962</v>
       </c>
       <c r="N5" t="n">
-        <v>14.19259157356192</v>
+        <v>14.18202189207348</v>
       </c>
       <c r="O5" t="n">
         <v>21.81518913779929</v>
       </c>
       <c r="P5" t="n">
-        <v>1.055176889417591</v>
+        <v>1.044607207929143</v>
       </c>
       <c r="Q5" t="n">
-        <v>311000000</v>
+        <v>340000000</v>
       </c>
       <c r="R5" t="n">
-        <v>2652.411575562701</v>
+        <v>2391.176470588235</v>
       </c>
       <c r="S5" t="n">
         <v>1</v>
       </c>
       <c r="T5" t="n">
-        <v>-0.1894280612981443</v>
+        <v>-0.1664560201963929</v>
       </c>
     </row>
     <row r="6">
@@ -899,7 +899,7 @@
         <v>1</v>
       </c>
       <c r="T6" t="n">
-        <v>-0.1863387520057622</v>
+        <v>-0.1656021193681139</v>
       </c>
     </row>
     <row r="7">
@@ -910,31 +910,31 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2007</t>
+          <t>2014</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Production and processing of metals</t>
+          <t>Chemical industry</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>voestalpine Stahl GmbH</t>
+          <t>Sandoz GmbH</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Carbon dioxide (CO2)</t>
+          <t>Hydrochlorofluorocarbons (HCFCs)</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>8730000000</v>
+        <v>623</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -945,37 +945,37 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>22.89003120691247</v>
+        <v>6.436150368369428</v>
       </c>
       <c r="K7" t="n">
         <v>19.08593942191924</v>
       </c>
       <c r="L7" t="n">
-        <v>3.804091784993233</v>
+        <v>-12.64978905354981</v>
       </c>
       <c r="M7" t="n">
-        <v>8.677774453654962</v>
+        <v>12.19095120020471</v>
       </c>
       <c r="N7" t="n">
-        <v>14.21225675325751</v>
+        <v>-5.754800831835284</v>
       </c>
       <c r="O7" t="n">
-        <v>21.81518913779929</v>
+        <v>12.83601552677931</v>
       </c>
       <c r="P7" t="n">
-        <v>1.074842069113174</v>
+        <v>-6.399865158409884</v>
       </c>
       <c r="Q7" t="n">
-        <v>329000000</v>
+        <v>10</v>
       </c>
       <c r="R7" t="n">
-        <v>2553.495440729484</v>
+        <v>6130</v>
       </c>
       <c r="S7" t="n">
         <v>1</v>
       </c>
       <c r="T7" t="n">
-        <v>-0.1853117660132111</v>
+        <v>-0.1534878890415876</v>
       </c>
     </row>
     <row r="8">
@@ -986,22 +986,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2010</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Production and processing of metals</t>
+          <t>Energy sector</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>voestalpine Stahl GmbH</t>
+          <t>WIEN ENERGIE GmbH</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1010,7 +1010,7 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>8810000000</v>
+        <v>1960000000</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -1021,37 +1021,37 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>22.89915327700801</v>
+        <v>21.39621031069904</v>
       </c>
       <c r="K8" t="n">
         <v>19.08593942191924</v>
       </c>
       <c r="L8" t="n">
-        <v>3.813213855088772</v>
+        <v>2.310270888779804</v>
       </c>
       <c r="M8" t="n">
-        <v>8.677774453654962</v>
+        <v>13.27250775700296</v>
       </c>
       <c r="N8" t="n">
-        <v>14.22137882335305</v>
+        <v>8.123702553696077</v>
       </c>
       <c r="O8" t="n">
-        <v>21.81518913779929</v>
+        <v>18.95130900089689</v>
       </c>
       <c r="P8" t="n">
-        <v>1.083964139208714</v>
+        <v>2.444901309802152</v>
       </c>
       <c r="Q8" t="n">
-        <v>330000000</v>
+        <v>192000000</v>
       </c>
       <c r="R8" t="n">
-        <v>2569.69696969697</v>
+        <v>920.8333333333334</v>
       </c>
       <c r="S8" t="n">
         <v>1</v>
       </c>
       <c r="T8" t="n">
-        <v>-0.1853117660132111</v>
+        <v>-0.08099240048918432</v>
       </c>
     </row>
     <row r="9">
@@ -1062,7 +1062,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2011</t>
+          <t>2018</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1082,52 +1082,52 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Carbon dioxide (CO2)</t>
+          <t>PCDD + PCDF (dioxins + furans) (as Teq)</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>8470000000</v>
+        <v>0.00087</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Regulated Climate/Ozone Risk - Global Environmental Impact</t>
+          <t>Critical Risk - Immediate Toxicity &amp; Severe Health Damage</t>
         </is>
       </c>
       <c r="I9" t="b">
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>22.85979634572844</v>
+        <v>0.0008696217693578752</v>
       </c>
       <c r="K9" t="n">
-        <v>19.08593942191924</v>
+        <v>3.796006532848082</v>
       </c>
       <c r="L9" t="n">
-        <v>3.773856923809202</v>
+        <v>-3.795136911078724</v>
       </c>
       <c r="M9" t="n">
         <v>8.677774453654962</v>
       </c>
       <c r="N9" t="n">
-        <v>14.18202189207348</v>
+        <v>-8.676904831885604</v>
       </c>
       <c r="O9" t="n">
-        <v>21.81518913779929</v>
+        <v>5.398162701517752</v>
       </c>
       <c r="P9" t="n">
-        <v>1.044607207929143</v>
+        <v>-5.397293079748395</v>
       </c>
       <c r="Q9" t="n">
-        <v>340000000</v>
+        <v>0.00125</v>
       </c>
       <c r="R9" t="n">
-        <v>2391.176470588235</v>
+        <v>-30.4</v>
       </c>
       <c r="S9" t="n">
         <v>1</v>
       </c>
       <c r="T9" t="n">
-        <v>-0.1827503727036507</v>
+        <v>-0.06713502783025438</v>
       </c>
     </row>
     <row r="10">
@@ -1158,52 +1158,52 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Carbon dioxide (CO2)</t>
+          <t>PCDD + PCDF (dioxins + furans) (as Teq)</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>6880000000</v>
+        <v>0.00137</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Regulated Climate/Ozone Risk - Global Environmental Impact</t>
+          <t>Critical Risk - Immediate Toxicity &amp; Severe Health Damage</t>
         </is>
       </c>
       <c r="I10" t="b">
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>22.65188448903701</v>
+        <v>0.001369062406237942</v>
       </c>
       <c r="K10" t="n">
-        <v>19.08593942191924</v>
+        <v>3.796006532848082</v>
       </c>
       <c r="L10" t="n">
-        <v>3.565945067117777</v>
+        <v>-3.794637470441844</v>
       </c>
       <c r="M10" t="n">
         <v>8.677774453654962</v>
       </c>
       <c r="N10" t="n">
-        <v>13.97411003538205</v>
+        <v>-8.676405391248723</v>
       </c>
       <c r="O10" t="n">
-        <v>21.81518913779929</v>
+        <v>5.398162701517752</v>
       </c>
       <c r="P10" t="n">
-        <v>0.8366953512377187</v>
+        <v>-5.396793639111515</v>
       </c>
       <c r="Q10" t="n">
-        <v>259000000</v>
+        <v>0.00176</v>
       </c>
       <c r="R10" t="n">
-        <v>2556.370656370656</v>
+        <v>-22.15909090909092</v>
       </c>
       <c r="S10" t="n">
         <v>1</v>
       </c>
       <c r="T10" t="n">
-        <v>-0.1827382704483099</v>
+        <v>-0.06190467497102337</v>
       </c>
     </row>
     <row r="11">
@@ -1214,7 +1214,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2015</t>
+          <t>2016</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1229,57 +1229,57 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>voestalpine Stahl GmbH</t>
+          <t>voestalpine Stahl Donawitz GmbH</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Carbon dioxide (CO2)</t>
+          <t>Cadmium and compounds (as Cd)</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>8640000000</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Regulated Climate/Ozone Risk - Global Environmental Impact</t>
+          <t>Critical Risk - Immediate Toxicity &amp; Severe Health Damage</t>
         </is>
       </c>
       <c r="I11" t="b">
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>22.87966841987812</v>
+        <v>4.429625613473161</v>
       </c>
       <c r="K11" t="n">
-        <v>19.08593942191924</v>
+        <v>3.796006532848082</v>
       </c>
       <c r="L11" t="n">
-        <v>3.79372899795888</v>
+        <v>0.6336190806250785</v>
       </c>
       <c r="M11" t="n">
         <v>8.677774453654962</v>
       </c>
       <c r="N11" t="n">
-        <v>14.20189396622315</v>
+        <v>-4.248148840181801</v>
       </c>
       <c r="O11" t="n">
-        <v>21.81518913779929</v>
+        <v>5.398162701517752</v>
       </c>
       <c r="P11" t="n">
-        <v>1.064479282078821</v>
+        <v>-0.9685370880445916</v>
       </c>
       <c r="Q11" t="n">
-        <v>366000000</v>
+        <v>16.2</v>
       </c>
       <c r="R11" t="n">
-        <v>2260.655737704918</v>
+        <v>411.7283950617284</v>
       </c>
       <c r="S11" t="n">
         <v>1</v>
       </c>
       <c r="T11" t="n">
-        <v>-0.179688116658861</v>
+        <v>-0.05561132410076264</v>
       </c>
     </row>
     <row r="12">
@@ -1305,57 +1305,55 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>voestalpine Stahl GmbH</t>
+          <t>voestalpine Stahl Donawitz GmbH</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Carbon dioxide (CO2)</t>
+          <t>PCDD + PCDF (dioxins + furans) (as Teq)</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>8600000000</v>
+        <v>0.00013</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Regulated Climate/Ozone Risk - Global Environmental Impact</t>
+          <t>Critical Risk - Immediate Toxicity &amp; Severe Health Damage</t>
         </is>
       </c>
       <c r="I12" t="b">
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>22.87502804032215</v>
+        <v>0.0001299915507322619</v>
       </c>
       <c r="K12" t="n">
-        <v>19.08593942191924</v>
+        <v>3.796006532848082</v>
       </c>
       <c r="L12" t="n">
-        <v>3.789088618402918</v>
+        <v>-3.79587654129735</v>
       </c>
       <c r="M12" t="n">
         <v>8.677774453654962</v>
       </c>
       <c r="N12" t="n">
-        <v>14.19725358666719</v>
+        <v>-8.677644462104229</v>
       </c>
       <c r="O12" t="n">
-        <v>21.81518913779929</v>
+        <v>5.398162701517752</v>
       </c>
       <c r="P12" t="n">
-        <v>1.059838902522859</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>362000000</v>
-      </c>
+        <v>-5.39803270996702</v>
+      </c>
+      <c r="Q12" t="inlineStr"/>
       <c r="R12" t="n">
-        <v>2275.690607734807</v>
+        <v>0</v>
       </c>
       <c r="S12" t="n">
         <v>1</v>
       </c>
       <c r="T12" t="n">
-        <v>-0.179178948158403</v>
+        <v>-0.05228851713830907</v>
       </c>
     </row>
     <row r="13">
@@ -1366,7 +1364,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2013</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1386,52 +1384,52 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Carbon dioxide (CO2)</t>
+          <t>PCDD + PCDF (dioxins + furans) (as Teq)</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>8600000000</v>
+        <v>0.00104</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Regulated Climate/Ozone Risk - Global Environmental Impact</t>
+          <t>Critical Risk - Immediate Toxicity &amp; Severe Health Damage</t>
         </is>
       </c>
       <c r="I13" t="b">
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>22.87502804032215</v>
+        <v>0.001039459574662445</v>
       </c>
       <c r="K13" t="n">
-        <v>19.08593942191924</v>
+        <v>3.796006532848082</v>
       </c>
       <c r="L13" t="n">
-        <v>3.789088618402918</v>
+        <v>-3.79496707327342</v>
       </c>
       <c r="M13" t="n">
         <v>8.677774453654962</v>
       </c>
       <c r="N13" t="n">
-        <v>14.19725358666719</v>
+        <v>-8.676734994080299</v>
       </c>
       <c r="O13" t="n">
-        <v>21.81518913779929</v>
+        <v>5.398162701517752</v>
       </c>
       <c r="P13" t="n">
-        <v>1.059838902522859</v>
+        <v>-5.39712324194309</v>
       </c>
       <c r="Q13" t="n">
-        <v>371000000</v>
+        <v>0.00095</v>
       </c>
       <c r="R13" t="n">
-        <v>2218.059299191375</v>
+        <v>9.473684210526306</v>
       </c>
       <c r="S13" t="n">
         <v>1</v>
       </c>
       <c r="T13" t="n">
-        <v>-0.17867012403787</v>
+        <v>-0.05214793868935375</v>
       </c>
     </row>
     <row r="14">
@@ -1442,72 +1440,72 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2014</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Production and processing of metals</t>
+          <t>Mineral industry</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>voestalpine Stahl GmbH</t>
+          <t>Holcim (Österreich) GmbH</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Carbon dioxide (CO2)</t>
+          <t>Mercury and compounds (as Hg)</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>8660000000</v>
+        <v>42</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Regulated Climate/Ozone Risk - Global Environmental Impact</t>
+          <t>Critical Risk - Immediate Toxicity &amp; Severe Health Damage</t>
         </is>
       </c>
       <c r="I14" t="b">
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>22.88198055963623</v>
+        <v>3.761200115693562</v>
       </c>
       <c r="K14" t="n">
-        <v>19.08593942191924</v>
+        <v>3.796006532848082</v>
       </c>
       <c r="L14" t="n">
-        <v>3.796041137716994</v>
+        <v>-0.03480641715451993</v>
       </c>
       <c r="M14" t="n">
-        <v>8.677774453654962</v>
+        <v>12.68230993011178</v>
       </c>
       <c r="N14" t="n">
-        <v>14.20420610598127</v>
+        <v>-8.921109814418223</v>
       </c>
       <c r="O14" t="n">
-        <v>21.81518913779929</v>
+        <v>3.08644493453506</v>
       </c>
       <c r="P14" t="n">
-        <v>1.066791421836935</v>
+        <v>0.6747551811585022</v>
       </c>
       <c r="Q14" t="n">
-        <v>370000000</v>
+        <v>13.9</v>
       </c>
       <c r="R14" t="n">
-        <v>2240.540540540541</v>
+        <v>202.1582733812949</v>
       </c>
       <c r="S14" t="n">
         <v>1</v>
       </c>
       <c r="T14" t="n">
-        <v>-0.17867012403787</v>
+        <v>-0.04761595616081582</v>
       </c>
     </row>
     <row r="15">
@@ -1518,7 +1516,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2014</t>
+          <t>2013</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1533,16 +1531,16 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Sandoz GmbH</t>
+          <t>Borealis Polyolefine GmbH</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Hydrochlorofluorocarbons (HCFCs)</t>
+          <t>Hydro-fluorocarbons (HFCS)</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>623</v>
+        <v>108</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -1553,37 +1551,35 @@
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>6.436150368369428</v>
+        <v>4.691347882229143</v>
       </c>
       <c r="K15" t="n">
         <v>19.08593942191924</v>
       </c>
       <c r="L15" t="n">
-        <v>-12.64978905354981</v>
+        <v>-14.39459153969009</v>
       </c>
       <c r="M15" t="n">
         <v>12.19095120020471</v>
       </c>
       <c r="N15" t="n">
-        <v>-5.754800831835284</v>
+        <v>-7.499603317975568</v>
       </c>
       <c r="O15" t="n">
         <v>12.83601552677931</v>
       </c>
       <c r="P15" t="n">
-        <v>-6.399865158409884</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>10</v>
-      </c>
+        <v>-8.144667644550168</v>
+      </c>
+      <c r="Q15" t="inlineStr"/>
       <c r="R15" t="n">
-        <v>6130</v>
+        <v>0</v>
       </c>
       <c r="S15" t="n">
         <v>1</v>
       </c>
       <c r="T15" t="n">
-        <v>-0.1624277032504617</v>
+        <v>-0.03912153352872916</v>
       </c>
     </row>
     <row r="16">
@@ -1594,7 +1590,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2014</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1609,16 +1605,16 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Sandoz GmbH</t>
+          <t>Patheon Austria GmbH &amp; CoKG</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Hydrochlorofluorocarbons (HCFCs)</t>
+          <t>Hydro-fluorocarbons (HFCS)</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>10</v>
+        <v>144</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -1629,37 +1625,37 @@
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>2.397895272798371</v>
+        <v>4.976733742420574</v>
       </c>
       <c r="K16" t="n">
         <v>19.08593942191924</v>
       </c>
       <c r="L16" t="n">
-        <v>-16.68804414912086</v>
+        <v>-14.10920567949866</v>
       </c>
       <c r="M16" t="n">
         <v>12.19095120020471</v>
       </c>
       <c r="N16" t="n">
-        <v>-9.793055927406341</v>
+        <v>-7.214217457784137</v>
       </c>
       <c r="O16" t="n">
         <v>12.83601552677931</v>
       </c>
       <c r="P16" t="n">
-        <v>-10.43812025398094</v>
+        <v>-7.859281784358737</v>
       </c>
       <c r="Q16" t="n">
-        <v>341</v>
+        <v>268</v>
       </c>
       <c r="R16" t="n">
-        <v>-97.0674486803519</v>
+        <v>-46.26865671641791</v>
       </c>
       <c r="S16" t="n">
         <v>1</v>
       </c>
       <c r="T16" t="n">
-        <v>-0.1294002393881796</v>
+        <v>-0.03729867326555114</v>
       </c>
     </row>
     <row r="17">
@@ -1670,72 +1666,72 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2011</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Mineral industry</t>
+          <t>Chemical industry</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Leube Zement GmbH</t>
+          <t>Borealis Polyolefine GmbH</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Naphthalene</t>
+          <t>Hydrochlorofluorocarbons (HCFCs)</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>1140</v>
+        <v>126</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>High Risk - Persistent Toxins, Carcinogens &amp; Long-Term Illness</t>
+          <t>Regulated Climate/Ozone Risk - Global Environmental Impact</t>
         </is>
       </c>
       <c r="I17" t="b">
         <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>7.039660349862076</v>
+        <v>4.844187086458591</v>
       </c>
       <c r="K17" t="n">
-        <v>4.923617305492665</v>
+        <v>19.08593942191924</v>
       </c>
       <c r="L17" t="n">
-        <v>2.116043044369411</v>
+        <v>-14.24175233546064</v>
       </c>
       <c r="M17" t="n">
-        <v>12.68230993011178</v>
+        <v>12.19095120020471</v>
       </c>
       <c r="N17" t="n">
-        <v>-5.642649580249709</v>
+        <v>-7.34676411374612</v>
       </c>
       <c r="O17" t="n">
-        <v>4.870484311519177</v>
+        <v>12.83601552677931</v>
       </c>
       <c r="P17" t="n">
-        <v>2.169176038342899</v>
+        <v>-7.99182844032072</v>
       </c>
       <c r="Q17" t="n">
-        <v>101</v>
+        <v>167</v>
       </c>
       <c r="R17" t="n">
-        <v>1028.712871287129</v>
+        <v>-24.55089820359281</v>
       </c>
       <c r="S17" t="n">
         <v>1</v>
       </c>
       <c r="T17" t="n">
-        <v>-0.1024886395961313</v>
+        <v>-0.0310181415716172</v>
       </c>
     </row>
     <row r="18">
@@ -1746,7 +1742,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2010</t>
+          <t>2009</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1761,16 +1757,16 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Patheon Austria GmbH &amp; Co KG</t>
+          <t>Sandoz GmbH</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Hydrochlorofluorocarbons (HCFCs)</t>
+          <t>Hydro-fluorocarbons (HFCS)</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>36</v>
+        <v>351</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -1781,37 +1777,37 @@
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>3.610917912644224</v>
+        <v>5.863631175598097</v>
       </c>
       <c r="K18" t="n">
         <v>19.08593942191924</v>
       </c>
       <c r="L18" t="n">
-        <v>-15.47502150927501</v>
+        <v>-13.22230824632114</v>
       </c>
       <c r="M18" t="n">
         <v>12.19095120020471</v>
       </c>
       <c r="N18" t="n">
-        <v>-8.580033287560488</v>
+        <v>-6.327320024606615</v>
       </c>
       <c r="O18" t="n">
         <v>12.83601552677931</v>
       </c>
       <c r="P18" t="n">
-        <v>-9.225097614135088</v>
+        <v>-6.972384351181215</v>
       </c>
       <c r="Q18" t="n">
-        <v>600</v>
+        <v>242</v>
       </c>
       <c r="R18" t="n">
-        <v>-94</v>
+        <v>45.04132231404959</v>
       </c>
       <c r="S18" t="n">
         <v>1</v>
       </c>
       <c r="T18" t="n">
-        <v>-0.1021735843681947</v>
+        <v>-0.03074069332998075</v>
       </c>
     </row>
     <row r="19">
@@ -1822,31 +1818,31 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2010</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Energy sector</t>
+          <t>Chemical industry</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>OMV Downstream GmbH</t>
+          <t>Patheon Austria GmbH &amp; CoKG</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Hydrochlorofluorocarbons (HCFCs)</t>
+          <t>Hydro-fluorocarbons (HFCS)</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>147</v>
+        <v>122</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -1857,37 +1853,37 @@
         <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>4.997212273764115</v>
+        <v>4.812184355372417</v>
       </c>
       <c r="K19" t="n">
         <v>19.08593942191924</v>
       </c>
       <c r="L19" t="n">
-        <v>-14.08872714815512</v>
+        <v>-14.27375506654682</v>
       </c>
       <c r="M19" t="n">
-        <v>13.27250775700296</v>
+        <v>12.19095120020471</v>
       </c>
       <c r="N19" t="n">
-        <v>-8.275295483238848</v>
+        <v>-7.378766844832295</v>
       </c>
       <c r="O19" t="n">
-        <v>18.95130900089689</v>
+        <v>12.83601552677931</v>
       </c>
       <c r="P19" t="n">
-        <v>-13.95409672713277</v>
+        <v>-8.023831171406894</v>
       </c>
       <c r="Q19" t="n">
-        <v>345</v>
+        <v>144</v>
       </c>
       <c r="R19" t="n">
-        <v>-57.39130434782609</v>
+        <v>-15.27777777777778</v>
       </c>
       <c r="S19" t="n">
         <v>1</v>
       </c>
       <c r="T19" t="n">
-        <v>-0.09401107019937116</v>
+        <v>-0.03011600583653051</v>
       </c>
     </row>
     <row r="20">
@@ -1898,7 +1894,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2010</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1922,7 +1918,7 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>1960000000</v>
+        <v>1150000000</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -1933,37 +1929,37 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>21.39621031069904</v>
+        <v>20.86302778019114</v>
       </c>
       <c r="K20" t="n">
         <v>19.08593942191924</v>
       </c>
       <c r="L20" t="n">
-        <v>2.310270888779804</v>
+        <v>1.7770883582719</v>
       </c>
       <c r="M20" t="n">
         <v>13.27250775700296</v>
       </c>
       <c r="N20" t="n">
-        <v>8.123702553696077</v>
+        <v>7.590520023188173</v>
       </c>
       <c r="O20" t="n">
         <v>18.95130900089689</v>
       </c>
       <c r="P20" t="n">
-        <v>2.444901309802152</v>
+        <v>1.911718779294247</v>
       </c>
       <c r="Q20" t="n">
-        <v>192000000</v>
+        <v>174000000</v>
       </c>
       <c r="R20" t="n">
-        <v>920.8333333333334</v>
+        <v>560.9195402298851</v>
       </c>
       <c r="S20" t="n">
         <v>1</v>
       </c>
       <c r="T20" t="n">
-        <v>-0.08997761986909603</v>
+        <v>-0.02813035744711045</v>
       </c>
     </row>
     <row r="21">
@@ -1974,31 +1970,31 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2013</t>
+          <t>2008</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Chemical industry</t>
+          <t>Energy sector</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Patheon Austria GmbH &amp; Co KG</t>
+          <t>EVN AG</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Hydrochlorofluorocarbons (HCFCs)</t>
+          <t>Carbon dioxide (CO2)</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>25</v>
+        <v>968000000</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -2009,37 +2005,37 @@
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>3.258096538021482</v>
+        <v>20.69074264627391</v>
       </c>
       <c r="K21" t="n">
         <v>19.08593942191924</v>
       </c>
       <c r="L21" t="n">
-        <v>-15.82784288389775</v>
+        <v>1.604803224354672</v>
       </c>
       <c r="M21" t="n">
-        <v>12.19095120020471</v>
+        <v>13.27250775700296</v>
       </c>
       <c r="N21" t="n">
-        <v>-8.93285466218323</v>
+        <v>7.418234889270945</v>
       </c>
       <c r="O21" t="n">
-        <v>12.83601552677931</v>
+        <v>18.95130900089689</v>
       </c>
       <c r="P21" t="n">
-        <v>-9.57791898875783</v>
+        <v>1.739433645377019</v>
       </c>
       <c r="Q21" t="n">
-        <v>41</v>
+        <v>142000000</v>
       </c>
       <c r="R21" t="n">
-        <v>-39.02439024390244</v>
+        <v>581.6901408450703</v>
       </c>
       <c r="S21" t="n">
         <v>1</v>
       </c>
       <c r="T21" t="n">
-        <v>-0.08864713343244413</v>
+        <v>-0.02489183351532764</v>
       </c>
     </row>
   </sheetData>
@@ -2053,7 +2049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2075,7 +2071,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>87</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3">
@@ -2085,7 +2081,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>46</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4">
@@ -2095,7 +2091,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>22</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -2105,7 +2101,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -2115,16 +2111,6 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Other activities</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2139,7 +2125,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2161,37 +2147,27 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>96</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Moderate Risk - Air Pollution, Corrosives &amp; Community Exposure</t>
+          <t>Critical Risk - Immediate Toxicity &amp; Severe Health Damage</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>42</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Critical Risk - Immediate Toxicity &amp; Severe Health Damage</t>
+          <t>Moderate Risk - Air Pollution, Corrosives &amp; Community Exposure</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>High Risk - Persistent Toxins, Carcinogens &amp; Long-Term Illness</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -2205,7 +2181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2237,7 +2213,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>46</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
@@ -2248,11 +2224,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Moderate Risk - Air Pollution, Corrosives &amp; Community Exposure</t>
+          <t>Regulated Climate/Ozone Risk - Global Environmental Impact</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>37</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -2267,7 +2243,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>28</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -2278,11 +2254,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Regulated Climate/Ozone Risk - Global Environmental Impact</t>
+          <t>Moderate Risk - Air Pollution, Corrosives &amp; Community Exposure</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>22</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
@@ -2297,96 +2273,36 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Waste and wastewater management</t>
+          <t>Mineral industry</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Regulated Climate/Ozone Risk - Global Environmental Impact</t>
+          <t>Critical Risk - Immediate Toxicity &amp; Severe Health Damage</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Mineral industry</t>
+          <t>Waste and wastewater management</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Critical Risk - Immediate Toxicity &amp; Severe Health Damage</t>
+          <t>Regulated Climate/Ozone Risk - Global Environmental Impact</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Mineral industry</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Moderate Risk - Air Pollution, Corrosives &amp; Community Exposure</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Energy sector</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Moderate Risk - Air Pollution, Corrosives &amp; Community Exposure</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Other activities</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Regulated Climate/Ozone Risk - Global Environmental Impact</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Mineral industry</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>High Risk - Persistent Toxins, Carcinogens &amp; Long-Term Illness</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>